<commit_message>
update SW version 18 Aug 2026
</commit_message>
<xml_diff>
--- a/web-console/server/assets/pdf_template.xlsx
+++ b/web-console/server/assets/pdf_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\DEV\UBA6\web-console\server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A869A33E-9D32-4A31-9FF6-D76A159C517A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FDEBAEB-E12F-4A4F-92EF-492B61E60570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3E3B58E4-0181-4207-8002-E1D914CEBC2E}"/>
   </bookViews>
@@ -196,83 +196,19 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="7">
+  <borders count="1">
     <border>
       <left/>
       <right/>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -282,33 +218,22 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
@@ -316,9 +241,6 @@
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5730,7 +5652,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="605922" y="396588"/>
+          <a:off x="605922" y="380713"/>
           <a:ext cx="9312753" cy="4137009"/>
           <a:chOff x="614350" y="401783"/>
           <a:chExt cx="9325165" cy="4265799"/>
@@ -6193,7 +6115,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:O100"/>
+  <dimension ref="B2:O78"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.44140625" style="2" customWidth="1"/>
@@ -6202,908 +6124,665 @@
     <col min="4" max="9" width="19.6640625" style="2" customWidth="1"/>
     <col min="10" max="10" width="9.44140625" style="2" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="4.109375" style="2" customWidth="1"/>
-    <col min="12" max="12" width="9.109375" style="15"/>
+    <col min="12" max="12" width="9.109375" style="8"/>
     <col min="13" max="13" width="82.44140625" style="2" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="123.33203125" style="2" customWidth="1"/>
     <col min="15" max="15" width="78.88671875" style="2" customWidth="1"/>
     <col min="16" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="J1" s="16"/>
-    </row>
     <row r="2" spans="2:14" ht="8.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="3"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="8"/>
-      <c r="K2" s="5"/>
+      <c r="J2" s="4"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B3" s="6"/>
-      <c r="D3" s="7" t="s">
+      <c r="B3" s="4"/>
+      <c r="D3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="8"/>
-      <c r="F3" s="7" t="s">
+      <c r="E3" s="4"/>
+      <c r="F3" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="J3" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="K3" s="9"/>
-      <c r="N3" s="10"/>
+      <c r="K3" s="4"/>
+      <c r="N3" s="5"/>
     </row>
     <row r="4" spans="2:14" ht="5.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="6"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="8"/>
-      <c r="I4" s="8"/>
-      <c r="J4" s="8"/>
-      <c r="K4" s="9"/>
-      <c r="N4" s="10"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
+      <c r="N4" s="5"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B5" s="12"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="18"/>
-      <c r="I5" s="18"/>
-      <c r="J5" s="18"/>
-      <c r="K5" s="13"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
     </row>
     <row r="6" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B6" s="12"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
-      <c r="I6" s="18"/>
-      <c r="J6" s="18"/>
-      <c r="K6" s="13"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B7" s="12"/>
-      <c r="C7" s="18"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="18"/>
-      <c r="H7" s="18"/>
-      <c r="I7" s="18"/>
-      <c r="J7" s="18"/>
-      <c r="K7" s="13"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B8" s="12"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="18"/>
-      <c r="H8" s="18"/>
-      <c r="I8" s="18"/>
-      <c r="J8" s="18"/>
-      <c r="K8" s="13"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="9"/>
+      <c r="J8" s="9"/>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B9" s="12"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="18"/>
-      <c r="H9" s="18"/>
-      <c r="I9" s="18"/>
-      <c r="J9" s="18"/>
-      <c r="K9" s="13"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="9"/>
+      <c r="J9" s="9"/>
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B10" s="12"/>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
-      <c r="G10" s="18"/>
-      <c r="H10" s="18"/>
-      <c r="I10" s="18"/>
-      <c r="J10" s="18"/>
-      <c r="K10" s="13"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="9"/>
+      <c r="J10" s="9"/>
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B11" s="12"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
-      <c r="G11" s="18"/>
-      <c r="H11" s="18"/>
-      <c r="I11" s="18"/>
-      <c r="J11" s="18"/>
-      <c r="K11" s="13"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="9"/>
+      <c r="J11" s="9"/>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B12" s="12"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
-      <c r="G12" s="18"/>
-      <c r="H12" s="18"/>
-      <c r="I12" s="18"/>
-      <c r="J12" s="18"/>
-      <c r="K12" s="13"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
+      <c r="I12" s="9"/>
+      <c r="J12" s="9"/>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B13" s="12"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="18"/>
-      <c r="I13" s="18"/>
-      <c r="J13" s="18"/>
-      <c r="K13" s="13"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
+      <c r="J13" s="9"/>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B14" s="12"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="18"/>
-      <c r="H14" s="18"/>
-      <c r="I14" s="18"/>
-      <c r="J14" s="18"/>
-      <c r="K14" s="13"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="9"/>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B15" s="12"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="18"/>
-      <c r="G15" s="18"/>
-      <c r="H15" s="18"/>
-      <c r="I15" s="18"/>
-      <c r="J15" s="18"/>
-      <c r="K15" s="13"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="9"/>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B16" s="12"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
-      <c r="G16" s="18"/>
-      <c r="H16" s="18"/>
-      <c r="I16" s="18"/>
-      <c r="J16" s="18"/>
-      <c r="K16" s="13"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="9"/>
+      <c r="J16" s="9"/>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B17" s="12"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="18"/>
-      <c r="G17" s="18"/>
-      <c r="H17" s="18"/>
-      <c r="I17" s="18"/>
-      <c r="J17" s="18"/>
-      <c r="K17" s="13"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+      <c r="I17" s="9"/>
+      <c r="J17" s="9"/>
     </row>
     <row r="18" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B18" s="12"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="18"/>
-      <c r="G18" s="18"/>
-      <c r="H18" s="18"/>
-      <c r="I18" s="18"/>
-      <c r="J18" s="18"/>
-      <c r="K18" s="13"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="9"/>
+      <c r="I18" s="9"/>
+      <c r="J18" s="9"/>
     </row>
     <row r="19" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B19" s="12"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="18"/>
-      <c r="F19" s="18"/>
-      <c r="G19" s="18"/>
-      <c r="H19" s="18"/>
-      <c r="I19" s="18"/>
-      <c r="J19" s="18"/>
-      <c r="K19" s="13"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="9"/>
+      <c r="J19" s="9"/>
     </row>
     <row r="20" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B20" s="12"/>
-      <c r="C20" s="18"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="18"/>
-      <c r="F20" s="18"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="18"/>
-      <c r="I20" s="18"/>
-      <c r="J20" s="18"/>
-      <c r="K20" s="13"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+      <c r="I20" s="9"/>
+      <c r="J20" s="9"/>
     </row>
     <row r="21" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B21" s="12"/>
-      <c r="C21" s="18"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="18"/>
-      <c r="F21" s="18"/>
-      <c r="G21" s="18"/>
-      <c r="H21" s="18"/>
-      <c r="I21" s="18"/>
-      <c r="J21" s="18"/>
-      <c r="K21" s="13"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
+      <c r="J21" s="9"/>
     </row>
     <row r="22" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B22" s="12"/>
-      <c r="C22" s="18"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="18"/>
-      <c r="F22" s="18"/>
-      <c r="G22" s="18"/>
-      <c r="H22" s="18"/>
-      <c r="I22" s="18"/>
-      <c r="J22" s="18"/>
-      <c r="K22" s="13"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="9"/>
+      <c r="J22" s="9"/>
     </row>
     <row r="23" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B23" s="12"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="18"/>
-      <c r="F23" s="18"/>
-      <c r="G23" s="18"/>
-      <c r="H23" s="18"/>
-      <c r="I23" s="18"/>
-      <c r="J23" s="18"/>
-      <c r="K23" s="13"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="9"/>
+      <c r="I23" s="9"/>
+      <c r="J23" s="9"/>
     </row>
     <row r="24" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B24" s="12"/>
-      <c r="C24" s="18"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="18"/>
-      <c r="F24" s="18"/>
-      <c r="G24" s="18"/>
-      <c r="H24" s="18"/>
-      <c r="I24" s="18"/>
-      <c r="J24" s="18"/>
-      <c r="K24" s="13"/>
+      <c r="C24" s="9"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
+      <c r="G24" s="9"/>
+      <c r="H24" s="9"/>
+      <c r="I24" s="9"/>
+      <c r="J24" s="9"/>
     </row>
     <row r="25" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B25" s="12"/>
-      <c r="C25" s="18"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="18"/>
-      <c r="F25" s="18"/>
-      <c r="G25" s="18"/>
-      <c r="H25" s="18"/>
-      <c r="I25" s="18"/>
-      <c r="J25" s="18"/>
-      <c r="K25" s="13"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="9"/>
+      <c r="I25" s="9"/>
+      <c r="J25" s="9"/>
     </row>
     <row r="26" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B26" s="12"/>
-      <c r="C26" s="18"/>
-      <c r="D26" s="18"/>
-      <c r="E26" s="18"/>
-      <c r="F26" s="18"/>
-      <c r="G26" s="18"/>
-      <c r="H26" s="18"/>
-      <c r="I26" s="18"/>
-      <c r="J26" s="18"/>
-      <c r="K26" s="13"/>
-      <c r="M26" s="14"/>
-    </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B27" s="12"/>
-      <c r="K27" s="13"/>
+      <c r="C26" s="9"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="9"/>
+      <c r="G26" s="9"/>
+      <c r="H26" s="9"/>
+      <c r="I26" s="9"/>
+      <c r="J26" s="9"/>
+      <c r="M26" s="7"/>
     </row>
     <row r="28" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B28" s="6"/>
-      <c r="D28" s="8" t="s">
+      <c r="B28" s="4"/>
+      <c r="K28" s="4"/>
+    </row>
+    <row r="29" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="D29" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E28" s="8"/>
-      <c r="F28" s="8"/>
-      <c r="G28" s="8"/>
-      <c r="H28" s="8" t="s">
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="I28" s="8"/>
-      <c r="J28" s="8"/>
-      <c r="K28" s="9"/>
-      <c r="L28" s="17"/>
-    </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B29" s="12"/>
-      <c r="D29" s="2" t="s">
+      <c r="I29" s="4"/>
+      <c r="J29" s="4"/>
+    </row>
+    <row r="30" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="D30" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H29" s="2" t="s">
+      <c r="H30" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I29" s="19"/>
-      <c r="K29" s="13"/>
-      <c r="L29" s="17"/>
-    </row>
-    <row r="30" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B30" s="12"/>
-      <c r="H30" s="2" t="s">
+      <c r="I30" s="10"/>
+      <c r="L30" s="4"/>
+      <c r="M30" s="4"/>
+      <c r="N30" s="4"/>
+      <c r="O30" s="4"/>
+    </row>
+    <row r="31" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="H31" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I30" s="19"/>
-      <c r="K30" s="13"/>
-      <c r="L30" s="6"/>
-      <c r="M30" s="8"/>
-      <c r="N30" s="8"/>
-      <c r="O30" s="8"/>
-    </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B31" s="12"/>
-      <c r="D31" s="2" t="s">
+      <c r="I31" s="10"/>
+      <c r="L31" s="4"/>
+      <c r="M31" s="4"/>
+      <c r="N31" s="4"/>
+      <c r="O31" s="4"/>
+    </row>
+    <row r="32" spans="2:15" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="D32" s="2" t="s">
         <v>12</v>
-      </c>
-      <c r="H31" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="I31" s="19"/>
-      <c r="K31" s="13"/>
-      <c r="L31" s="6"/>
-      <c r="M31" s="8"/>
-      <c r="N31" s="8"/>
-      <c r="O31" s="8"/>
-    </row>
-    <row r="32" spans="2:15" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="6"/>
-      <c r="D32" s="2" t="s">
-        <v>10</v>
       </c>
       <c r="E32" s="2"/>
       <c r="F32" s="2"/>
       <c r="G32" s="2"/>
       <c r="H32" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I32" s="10"/>
+      <c r="J32" s="2"/>
+    </row>
+    <row r="33" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="D33" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H33" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I32" s="19"/>
-      <c r="J32" s="2" t="s">
+      <c r="I33" s="10"/>
+      <c r="J33" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="K32" s="9"/>
-      <c r="L32" s="6"/>
-    </row>
-    <row r="33" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B33" s="12"/>
-      <c r="H33" s="2" t="s">
+      <c r="L33" s="4"/>
+      <c r="M33" s="4"/>
+      <c r="N33" s="4"/>
+      <c r="O33" s="4"/>
+    </row>
+    <row r="34" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="H34" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="I33" s="19"/>
-      <c r="J33" s="2" t="s">
+      <c r="I34" s="10"/>
+      <c r="J34" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="K33" s="13"/>
-      <c r="L33" s="6"/>
-      <c r="M33" s="8"/>
-      <c r="N33" s="8"/>
-      <c r="O33" s="8"/>
-    </row>
-    <row r="34" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B34" s="12"/>
-      <c r="H34" s="2" t="s">
+      <c r="L34" s="4"/>
+      <c r="M34" s="4"/>
+      <c r="N34" s="4"/>
+      <c r="O34" s="4"/>
+    </row>
+    <row r="35" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="H35" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="I34" s="19"/>
-      <c r="J34" s="2" t="s">
+      <c r="I35" s="10"/>
+      <c r="J35" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="K34" s="13"/>
-      <c r="L34" s="6"/>
-      <c r="M34" s="8"/>
-      <c r="N34" s="8"/>
-      <c r="O34" s="8"/>
-    </row>
-    <row r="35" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B35" s="12"/>
-      <c r="H35" s="2" t="s">
+      <c r="L35" s="4"/>
+      <c r="M35" s="4"/>
+      <c r="N35" s="4"/>
+      <c r="O35" s="4"/>
+    </row>
+    <row r="36" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="H36" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I35" s="19"/>
-      <c r="K35" s="13"/>
-      <c r="L35" s="6"/>
-      <c r="M35" s="8"/>
-      <c r="N35" s="8"/>
-      <c r="O35" s="8"/>
-    </row>
-    <row r="36" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B36" s="12"/>
-      <c r="D36" s="2" t="s">
+      <c r="I36" s="10"/>
+      <c r="L36" s="4"/>
+      <c r="M36" s="4"/>
+      <c r="N36" s="4"/>
+      <c r="O36" s="4"/>
+    </row>
+    <row r="37" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="D37" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="H36" s="2" t="s">
+      <c r="H37" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="I36" s="19"/>
-      <c r="K36" s="13"/>
-      <c r="L36" s="6"/>
-      <c r="M36" s="8"/>
-      <c r="N36" s="8"/>
-      <c r="O36" s="8"/>
-    </row>
-    <row r="37" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B37" s="12"/>
-      <c r="D37" s="2" t="s">
+      <c r="I37" s="10"/>
+      <c r="L37" s="4"/>
+      <c r="M37" s="4"/>
+      <c r="N37" s="4"/>
+      <c r="O37" s="4"/>
+    </row>
+    <row r="38" spans="3:15" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="D38" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H37" s="2" t="s">
+      <c r="E38" s="2"/>
+      <c r="F38" s="2"/>
+      <c r="G38" s="2"/>
+      <c r="H38" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="I37" s="19"/>
-      <c r="K37" s="13"/>
-      <c r="L37" s="6"/>
-      <c r="M37" s="8"/>
-      <c r="N37" s="8"/>
-      <c r="O37" s="8"/>
-    </row>
-    <row r="38" spans="2:15" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="6"/>
-      <c r="D38" s="8" t="s">
+      <c r="I38" s="10"/>
+      <c r="J38" s="2"/>
+    </row>
+    <row r="39" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="D39" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="K38" s="9"/>
-      <c r="L38" s="6"/>
-    </row>
-    <row r="39" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B39" s="12"/>
-      <c r="D39" s="21"/>
-      <c r="E39" s="21"/>
-      <c r="F39" s="21"/>
-      <c r="G39" s="21"/>
-      <c r="H39" s="21"/>
-      <c r="I39" s="21"/>
-      <c r="J39" s="21"/>
-      <c r="K39" s="13"/>
-      <c r="L39" s="6"/>
-      <c r="M39" s="8"/>
-      <c r="N39" s="8"/>
-      <c r="O39" s="8"/>
-    </row>
-    <row r="40" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B40" s="12"/>
-      <c r="K40" s="13"/>
-      <c r="L40" s="6"/>
-      <c r="M40" s="8"/>
-      <c r="N40" s="8"/>
-      <c r="O40" s="8"/>
-    </row>
-    <row r="41" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B41" s="12"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
+      <c r="G39" s="4"/>
+      <c r="H39" s="4"/>
+      <c r="I39" s="4"/>
+      <c r="J39" s="4"/>
+      <c r="L39" s="4"/>
+      <c r="M39" s="4"/>
+      <c r="N39" s="4"/>
+      <c r="O39" s="4"/>
+    </row>
+    <row r="40" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="L40" s="4"/>
+      <c r="M40" s="4"/>
+      <c r="N40" s="4"/>
+      <c r="O40" s="4"/>
+    </row>
+    <row r="41" spans="3:15" x14ac:dyDescent="0.3">
       <c r="C41" s="2">
         <v>1</v>
       </c>
-      <c r="D41" s="8"/>
-      <c r="G41" s="8"/>
-      <c r="H41" s="8" t="s">
+      <c r="D41" s="4"/>
+      <c r="G41" s="4"/>
+      <c r="H41" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I41" s="8"/>
-      <c r="J41" s="8"/>
-      <c r="K41" s="13"/>
-      <c r="L41" s="6"/>
-      <c r="M41" s="8"/>
-      <c r="N41" s="8"/>
-      <c r="O41" s="8"/>
-    </row>
-    <row r="42" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B42" s="12"/>
-      <c r="K42" s="13"/>
-      <c r="L42" s="6"/>
-      <c r="M42" s="8"/>
-      <c r="N42" s="8"/>
-      <c r="O42" s="8"/>
-    </row>
-    <row r="43" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B43" s="12"/>
-      <c r="K43" s="13"/>
-      <c r="L43" s="6"/>
-      <c r="M43" s="8"/>
-      <c r="N43" s="8"/>
-      <c r="O43" s="8"/>
-    </row>
-    <row r="44" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B44" s="12"/>
-      <c r="K44" s="13"/>
-      <c r="L44" s="6"/>
-      <c r="M44" s="8"/>
-      <c r="N44" s="8"/>
-      <c r="O44" s="8"/>
-    </row>
-    <row r="45" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B45" s="12"/>
-      <c r="K45" s="13"/>
-      <c r="L45" s="6"/>
-      <c r="M45" s="8"/>
-      <c r="N45" s="8"/>
-      <c r="O45" s="8"/>
-    </row>
-    <row r="46" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B46" s="12"/>
-      <c r="K46" s="13"/>
-      <c r="L46" s="6"/>
-      <c r="M46" s="8"/>
-      <c r="N46" s="8"/>
-      <c r="O46" s="8"/>
-    </row>
-    <row r="47" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B47" s="12"/>
-      <c r="K47" s="13"/>
-      <c r="L47" s="6"/>
-      <c r="M47" s="8"/>
-      <c r="N47" s="8"/>
-      <c r="O47" s="8"/>
-    </row>
-    <row r="48" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B48" s="12"/>
-      <c r="K48" s="13"/>
-      <c r="L48" s="6"/>
-      <c r="M48" s="8"/>
-      <c r="N48" s="8"/>
-      <c r="O48" s="8"/>
-    </row>
-    <row r="49" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B49" s="12"/>
-      <c r="K49" s="13"/>
-      <c r="L49" s="6"/>
-      <c r="M49" s="8"/>
-      <c r="N49" s="8"/>
-      <c r="O49" s="8"/>
-    </row>
-    <row r="50" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B50" s="12"/>
-      <c r="K50" s="13"/>
-      <c r="L50" s="6"/>
-      <c r="M50" s="8"/>
-      <c r="N50" s="8"/>
-      <c r="O50" s="8"/>
-    </row>
-    <row r="51" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B51" s="12"/>
-      <c r="K51" s="13"/>
-      <c r="L51" s="6"/>
-      <c r="M51" s="8"/>
-      <c r="N51" s="8"/>
-      <c r="O51" s="8"/>
-    </row>
-    <row r="52" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B52" s="12"/>
-      <c r="K52" s="13"/>
-      <c r="L52" s="6"/>
-      <c r="M52" s="8"/>
-      <c r="N52" s="8"/>
-      <c r="O52" s="8"/>
-    </row>
-    <row r="53" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B53" s="12"/>
-      <c r="K53" s="13"/>
-      <c r="L53" s="6"/>
-      <c r="M53" s="8"/>
-      <c r="N53" s="8"/>
-      <c r="O53" s="8"/>
-    </row>
-    <row r="54" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B54" s="12"/>
-      <c r="K54" s="13"/>
-      <c r="L54" s="6"/>
-      <c r="M54" s="8"/>
-      <c r="N54" s="8"/>
-      <c r="O54" s="8"/>
-    </row>
-    <row r="55" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B55" s="12"/>
-      <c r="K55" s="13"/>
-      <c r="L55" s="6"/>
-      <c r="M55" s="8"/>
-      <c r="N55" s="8"/>
-      <c r="O55" s="8"/>
-    </row>
-    <row r="56" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B56" s="12"/>
-      <c r="K56" s="13"/>
-      <c r="L56" s="6"/>
-      <c r="M56" s="8"/>
-      <c r="N56" s="8"/>
-      <c r="O56" s="8"/>
-    </row>
-    <row r="57" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B57" s="12"/>
-      <c r="K57" s="13"/>
-      <c r="L57" s="6"/>
-      <c r="M57" s="8"/>
-      <c r="N57" s="8"/>
-      <c r="O57" s="8"/>
-    </row>
-    <row r="58" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B58" s="12"/>
-      <c r="K58" s="13"/>
-      <c r="L58" s="6"/>
-      <c r="M58" s="8"/>
-      <c r="N58" s="8"/>
-      <c r="O58" s="8"/>
-    </row>
-    <row r="59" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B59" s="12"/>
-      <c r="K59" s="13"/>
-      <c r="L59" s="6"/>
-      <c r="M59" s="8"/>
-      <c r="N59" s="8"/>
-      <c r="O59" s="8"/>
-    </row>
-    <row r="60" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B60" s="12"/>
-      <c r="K60" s="13"/>
-      <c r="L60" s="6"/>
-      <c r="M60" s="8"/>
-      <c r="N60" s="8"/>
-      <c r="O60" s="8"/>
-    </row>
-    <row r="61" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B61" s="12"/>
-      <c r="K61" s="13"/>
-      <c r="L61" s="6"/>
-      <c r="M61" s="8"/>
-      <c r="N61" s="8"/>
-      <c r="O61" s="8"/>
-    </row>
-    <row r="62" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B62" s="12"/>
-      <c r="K62" s="13"/>
-      <c r="L62" s="6"/>
-      <c r="M62" s="8"/>
-      <c r="N62" s="8"/>
-      <c r="O62" s="8"/>
-    </row>
-    <row r="63" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B63" s="12"/>
-      <c r="K63" s="13"/>
-      <c r="L63" s="6"/>
-      <c r="M63" s="8"/>
-      <c r="N63" s="8"/>
-      <c r="O63" s="8"/>
-    </row>
-    <row r="64" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B64" s="12"/>
-      <c r="K64" s="13"/>
-      <c r="L64" s="6"/>
-      <c r="M64" s="8"/>
-      <c r="N64" s="8"/>
-      <c r="O64" s="8"/>
-    </row>
-    <row r="65" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B65" s="12"/>
-      <c r="K65" s="13"/>
-      <c r="L65" s="6"/>
-      <c r="M65" s="8"/>
-      <c r="N65" s="8"/>
-      <c r="O65" s="8"/>
-    </row>
-    <row r="66" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B66" s="12"/>
-      <c r="K66" s="13"/>
-      <c r="L66" s="6"/>
-      <c r="M66" s="8"/>
-      <c r="N66" s="8"/>
-      <c r="O66" s="8"/>
-    </row>
-    <row r="67" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B67" s="12"/>
-      <c r="K67" s="13"/>
-      <c r="L67" s="6"/>
-      <c r="M67" s="8"/>
-      <c r="N67" s="8"/>
-      <c r="O67" s="8"/>
-    </row>
-    <row r="68" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B68" s="12"/>
-      <c r="K68" s="13"/>
-      <c r="L68" s="6"/>
-      <c r="M68" s="8"/>
-      <c r="N68" s="8"/>
-      <c r="O68" s="8"/>
-    </row>
-    <row r="69" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B69" s="12"/>
-      <c r="K69" s="13"/>
-      <c r="L69" s="6"/>
-      <c r="M69" s="8"/>
-      <c r="N69" s="8"/>
-      <c r="O69" s="8"/>
-    </row>
-    <row r="70" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B70" s="12"/>
-      <c r="K70" s="13"/>
-      <c r="L70" s="6"/>
-      <c r="M70" s="8"/>
-      <c r="N70" s="8"/>
-      <c r="O70" s="8"/>
-    </row>
-    <row r="71" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B71" s="12"/>
-      <c r="K71" s="13"/>
-      <c r="L71" s="6"/>
-      <c r="M71" s="8"/>
-      <c r="N71" s="8"/>
-      <c r="O71" s="8"/>
-    </row>
-    <row r="72" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B72" s="12"/>
-      <c r="K72" s="13"/>
-      <c r="L72" s="6"/>
-      <c r="M72" s="8"/>
-      <c r="N72" s="8"/>
-      <c r="O72" s="8"/>
-    </row>
-    <row r="73" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B73" s="12"/>
-      <c r="K73" s="13"/>
-      <c r="L73" s="6"/>
-      <c r="M73" s="8"/>
-      <c r="N73" s="8"/>
-      <c r="O73" s="8"/>
-    </row>
-    <row r="74" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B74" s="12"/>
-      <c r="K74" s="13"/>
-      <c r="L74" s="6"/>
-      <c r="M74" s="8"/>
-      <c r="N74" s="8"/>
-      <c r="O74" s="8"/>
-    </row>
-    <row r="75" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B75" s="12"/>
-      <c r="K75" s="13"/>
-      <c r="L75" s="6"/>
-      <c r="M75" s="8"/>
-      <c r="N75" s="8"/>
-      <c r="O75" s="8"/>
-    </row>
-    <row r="76" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B76" s="12"/>
-      <c r="K76" s="13"/>
-      <c r="L76" s="6"/>
-      <c r="M76" s="8"/>
-      <c r="N76" s="8"/>
-      <c r="O76" s="8"/>
-    </row>
-    <row r="77" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B77" s="12"/>
-      <c r="K77" s="13"/>
-      <c r="L77" s="17"/>
-    </row>
-    <row r="78" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B78" s="12"/>
-      <c r="H78" s="8"/>
-      <c r="I78" s="8"/>
-      <c r="J78" s="8"/>
-      <c r="K78" s="13"/>
-    </row>
-    <row r="79" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B79" s="12"/>
-      <c r="K79" s="13"/>
-    </row>
-    <row r="80" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B80" s="12"/>
-      <c r="K80" s="13"/>
-    </row>
-    <row r="81" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B81" s="12"/>
-      <c r="K81" s="13"/>
-    </row>
-    <row r="82" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B82" s="12"/>
-      <c r="K82" s="13"/>
-    </row>
-    <row r="83" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B83" s="12"/>
-      <c r="K83" s="13"/>
-    </row>
-    <row r="84" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B84" s="12"/>
-      <c r="K84" s="13"/>
-    </row>
-    <row r="85" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B85" s="12"/>
-      <c r="K85" s="13"/>
-    </row>
-    <row r="86" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B86" s="12"/>
-      <c r="K86" s="13"/>
-    </row>
-    <row r="87" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B87" s="12"/>
-      <c r="K87" s="13"/>
-    </row>
-    <row r="88" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B88" s="12"/>
-      <c r="K88" s="13"/>
-    </row>
-    <row r="89" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B89" s="12"/>
-      <c r="K89" s="13"/>
-    </row>
-    <row r="90" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B90" s="12"/>
-      <c r="K90" s="13"/>
-    </row>
-    <row r="91" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B91" s="12"/>
-      <c r="K91" s="13"/>
-    </row>
-    <row r="92" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B92" s="12"/>
-      <c r="K92" s="13"/>
-    </row>
-    <row r="93" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B93" s="12"/>
-      <c r="K93" s="13"/>
-    </row>
-    <row r="94" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B94" s="12"/>
-      <c r="K94" s="13"/>
-    </row>
-    <row r="95" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B95" s="12"/>
-      <c r="K95" s="13"/>
-    </row>
-    <row r="96" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B96" s="12"/>
-      <c r="K96" s="13"/>
-    </row>
-    <row r="97" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B97" s="12"/>
-      <c r="K97" s="13"/>
-    </row>
-    <row r="98" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B98" s="12"/>
-      <c r="K98" s="13"/>
-    </row>
-    <row r="99" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B99" s="12"/>
-      <c r="K99" s="13"/>
-    </row>
-    <row r="100" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B100" s="12"/>
-      <c r="K100" s="13"/>
+      <c r="I41" s="4"/>
+      <c r="J41" s="4"/>
+      <c r="L41" s="4"/>
+      <c r="M41" s="4"/>
+      <c r="N41" s="4"/>
+      <c r="O41" s="4"/>
+    </row>
+    <row r="42" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="L42" s="4"/>
+      <c r="M42" s="4"/>
+      <c r="N42" s="4"/>
+      <c r="O42" s="4"/>
+    </row>
+    <row r="43" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="L43" s="4"/>
+      <c r="M43" s="4"/>
+      <c r="N43" s="4"/>
+      <c r="O43" s="4"/>
+    </row>
+    <row r="44" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="L44" s="4"/>
+      <c r="M44" s="4"/>
+      <c r="N44" s="4"/>
+      <c r="O44" s="4"/>
+    </row>
+    <row r="45" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="L45" s="4"/>
+      <c r="M45" s="4"/>
+      <c r="N45" s="4"/>
+      <c r="O45" s="4"/>
+    </row>
+    <row r="46" spans="3:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L46" s="4"/>
+      <c r="M46" s="4"/>
+      <c r="N46" s="4"/>
+      <c r="O46" s="4"/>
+    </row>
+    <row r="47" spans="3:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L47" s="4"/>
+      <c r="M47" s="4"/>
+      <c r="N47" s="4"/>
+      <c r="O47" s="4"/>
+    </row>
+    <row r="48" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="L48" s="4"/>
+      <c r="M48" s="4"/>
+      <c r="N48" s="4"/>
+      <c r="O48" s="4"/>
+    </row>
+    <row r="49" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L49" s="4"/>
+      <c r="M49" s="4"/>
+      <c r="N49" s="4"/>
+      <c r="O49" s="4"/>
+    </row>
+    <row r="50" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L50" s="4"/>
+      <c r="M50" s="4"/>
+      <c r="N50" s="4"/>
+      <c r="O50" s="4"/>
+    </row>
+    <row r="51" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L51" s="4"/>
+      <c r="M51" s="4"/>
+      <c r="N51" s="4"/>
+      <c r="O51" s="4"/>
+    </row>
+    <row r="52" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L52" s="4"/>
+      <c r="M52" s="4"/>
+      <c r="N52" s="4"/>
+      <c r="O52" s="4"/>
+    </row>
+    <row r="53" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L53" s="4"/>
+      <c r="M53" s="4"/>
+      <c r="N53" s="4"/>
+      <c r="O53" s="4"/>
+    </row>
+    <row r="54" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L54" s="4"/>
+      <c r="M54" s="4"/>
+      <c r="N54" s="4"/>
+      <c r="O54" s="4"/>
+    </row>
+    <row r="55" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L55" s="4"/>
+      <c r="M55" s="4"/>
+      <c r="N55" s="4"/>
+      <c r="O55" s="4"/>
+    </row>
+    <row r="56" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L56" s="4"/>
+      <c r="M56" s="4"/>
+      <c r="N56" s="4"/>
+      <c r="O56" s="4"/>
+    </row>
+    <row r="57" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L57" s="4"/>
+      <c r="M57" s="4"/>
+      <c r="N57" s="4"/>
+      <c r="O57" s="4"/>
+    </row>
+    <row r="58" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L58" s="4"/>
+      <c r="M58" s="4"/>
+      <c r="N58" s="4"/>
+      <c r="O58" s="4"/>
+    </row>
+    <row r="59" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L59" s="4"/>
+      <c r="M59" s="4"/>
+      <c r="N59" s="4"/>
+      <c r="O59" s="4"/>
+    </row>
+    <row r="60" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L60" s="4"/>
+      <c r="M60" s="4"/>
+      <c r="N60" s="4"/>
+      <c r="O60" s="4"/>
+    </row>
+    <row r="61" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L61" s="4"/>
+      <c r="M61" s="4"/>
+      <c r="N61" s="4"/>
+      <c r="O61" s="4"/>
+    </row>
+    <row r="62" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L62" s="4"/>
+      <c r="M62" s="4"/>
+      <c r="N62" s="4"/>
+      <c r="O62" s="4"/>
+    </row>
+    <row r="63" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L63" s="4"/>
+      <c r="M63" s="4"/>
+      <c r="N63" s="4"/>
+      <c r="O63" s="4"/>
+    </row>
+    <row r="64" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L64" s="4"/>
+      <c r="M64" s="4"/>
+      <c r="N64" s="4"/>
+      <c r="O64" s="4"/>
+    </row>
+    <row r="65" spans="8:15" x14ac:dyDescent="0.3">
+      <c r="L65" s="4"/>
+      <c r="M65" s="4"/>
+      <c r="N65" s="4"/>
+      <c r="O65" s="4"/>
+    </row>
+    <row r="66" spans="8:15" x14ac:dyDescent="0.3">
+      <c r="L66" s="4"/>
+      <c r="M66" s="4"/>
+      <c r="N66" s="4"/>
+      <c r="O66" s="4"/>
+    </row>
+    <row r="67" spans="8:15" x14ac:dyDescent="0.3">
+      <c r="L67" s="4"/>
+      <c r="M67" s="4"/>
+      <c r="N67" s="4"/>
+      <c r="O67" s="4"/>
+    </row>
+    <row r="68" spans="8:15" x14ac:dyDescent="0.3">
+      <c r="L68" s="4"/>
+      <c r="M68" s="4"/>
+      <c r="N68" s="4"/>
+      <c r="O68" s="4"/>
+    </row>
+    <row r="69" spans="8:15" x14ac:dyDescent="0.3">
+      <c r="L69" s="4"/>
+      <c r="M69" s="4"/>
+      <c r="N69" s="4"/>
+      <c r="O69" s="4"/>
+    </row>
+    <row r="70" spans="8:15" x14ac:dyDescent="0.3">
+      <c r="L70" s="4"/>
+      <c r="M70" s="4"/>
+      <c r="N70" s="4"/>
+      <c r="O70" s="4"/>
+    </row>
+    <row r="71" spans="8:15" x14ac:dyDescent="0.3">
+      <c r="L71" s="4"/>
+      <c r="M71" s="4"/>
+      <c r="N71" s="4"/>
+      <c r="O71" s="4"/>
+    </row>
+    <row r="72" spans="8:15" x14ac:dyDescent="0.3">
+      <c r="L72" s="4"/>
+      <c r="M72" s="4"/>
+      <c r="N72" s="4"/>
+      <c r="O72" s="4"/>
+    </row>
+    <row r="73" spans="8:15" x14ac:dyDescent="0.3">
+      <c r="L73" s="4"/>
+      <c r="M73" s="4"/>
+      <c r="N73" s="4"/>
+      <c r="O73" s="4"/>
+    </row>
+    <row r="74" spans="8:15" x14ac:dyDescent="0.3">
+      <c r="L74" s="4"/>
+      <c r="M74" s="4"/>
+      <c r="N74" s="4"/>
+      <c r="O74" s="4"/>
+    </row>
+    <row r="75" spans="8:15" x14ac:dyDescent="0.3">
+      <c r="L75" s="4"/>
+      <c r="M75" s="4"/>
+      <c r="N75" s="4"/>
+      <c r="O75" s="4"/>
+    </row>
+    <row r="76" spans="8:15" x14ac:dyDescent="0.3">
+      <c r="L76" s="4"/>
+      <c r="M76" s="4"/>
+      <c r="N76" s="4"/>
+      <c r="O76" s="4"/>
+    </row>
+    <row r="78" spans="8:15" x14ac:dyDescent="0.3">
+      <c r="H78" s="4"/>
+      <c r="I78" s="4"/>
+      <c r="J78" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="D39:J39"/>
-  </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="8" scale="49" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="57" fitToHeight="72" orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;LUBA Test Report&amp;R&amp;D</oddHeader>
+    <oddFooter>Page &amp;P of &amp;N</oddFooter>
+  </headerFooter>
+  <rowBreaks count="2" manualBreakCount="2">
+    <brk id="41" max="11" man="1"/>
+    <brk id="75" max="11" man="1"/>
+  </rowBreaks>
+  <colBreaks count="1" manualBreakCount="1">
+    <brk id="3" max="149" man="1"/>
+  </colBreaks>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
@@ -7123,25 +6802,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="11" t="s">
         <v>23</v>
       </c>
       <c r="B1" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="C1" s="11" t="s">
         <v>22</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="E1" s="11" t="s">
         <v>24</v>
       </c>
       <c r="F1" t="s">
         <v>26</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="G1" s="11" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>